<commit_message>
fix: interval modbus tcp fl setting
</commit_message>
<xml_diff>
--- a/summary/summary report.xlsx
+++ b/summary/summary report.xlsx
@@ -125,8 +125,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TorqueSummary" displayName="TorqueSummary" ref="A1:T2" headerRowCount="1">
-  <autoFilter ref="A1:T2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TorqueSummary" displayName="TorqueSummary" ref="A1:T7" headerRowCount="1">
+  <autoFilter ref="A1:T7"/>
   <tableColumns count="20">
     <tableColumn id="1" name="Saved At"/>
     <tableColumn id="2" name="Date"/>
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T2"/>
+  <dimension ref="A1:T7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -590,7 +590,6 @@
           <t>Inner Tie Rod</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
         <v>1</v>
       </c>
@@ -609,7 +608,6 @@
           <t>S/Link #1</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
         <v>-29.999996</v>
       </c>
@@ -624,7 +622,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
           <t>260622-B-PARTNO-S-PM-01-04.csv</t>
@@ -638,6 +635,354 @@
       <c r="T2" t="inlineStr">
         <is>
           <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/report\260622-B-PARTNO-S-PM-01-04.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-23 13:30:59</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Breakaway Torque</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Inner Tie Rod</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Setting (S)</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>S/Link #1</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>-29.999996</v>
+      </c>
+      <c r="L3" t="n">
+        <v>29.999998</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.010935</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>260623-B-PARTNO-S-PM-01.csv</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/csv\260623-B-PARTNO-S-PM-01.csv</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/report\260623-B-PARTNO-S-PM-01.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-23 13:31:04</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Breakaway Torque</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Inner Tie Rod</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Setting (S)</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>S/Link #1</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>-29.999996</v>
+      </c>
+      <c r="L4" t="n">
+        <v>29.999998</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.010935</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>260623-B-PARTNO-S-PM-01.csv</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/csv\260623-B-PARTNO-S-PM-01.csv</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/report\260623-B-PARTNO-S-PM-01.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-23 13:31:08</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Breakaway Torque</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Inner Tie Rod</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Setting (S)</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>S/Link #1</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>-29.999996</v>
+      </c>
+      <c r="L5" t="n">
+        <v>29.999998</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.010935</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>260623-B-PARTNO-S-PM-01.csv</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/csv\260623-B-PARTNO-S-PM-01.csv</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/report\260623-B-PARTNO-S-PM-01.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-06-23 13:37:40</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Breakaway Torque</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Inner Tie Rod</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Development (D)</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>S/Link #1</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>-29.999996</v>
+      </c>
+      <c r="L6" t="n">
+        <v>29.999998</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.010935</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>260623-B-PARTNO-D-PM-01-01.csv</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/csv\260623-B-PARTNO-D-PM-01-01.csv</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/report\260623-B-PARTNO-D-PM-01-01.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-06-23 13:37:43</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Breakaway Torque</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Inner Tie Rod</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Development (D)</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>S/Link #1</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="n">
+        <v>-29.999996</v>
+      </c>
+      <c r="L7" t="n">
+        <v>29.999998</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0.010935</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>260623-B-PARTNO-D-PM-01-02.csv</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/csv\260623-B-PARTNO-D-PM-01-02.csv</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>D:/DuAn/18.Other/plot_draw/plot_ZE-SG3/report\260623-B-PARTNO-D-PM-01-02.xlsx</t>
         </is>
       </c>
     </row>

</xml_diff>